<commit_message>
Portfolio page+ Edit Page + Share Page
Added:
- Portfolio page (as Section to Home page)
- News page (as Section to Home page) (just ignore it so far)
- Edit page & Create page
- Share page
</commit_message>
<xml_diff>
--- a/time-table.xlsx
+++ b/time-table.xlsx
@@ -39,9 +39,6 @@
     <t>Login page</t>
   </si>
   <si>
-    <t>Dashboard</t>
-  </si>
-  <si>
     <t>Constructor</t>
   </si>
   <si>
@@ -61,6 +58,9 @@
   </si>
   <si>
     <t>General time on development:</t>
+  </si>
+  <si>
+    <t>Dashboard(WIP)</t>
   </si>
 </sst>
 </file>
@@ -439,13 +439,13 @@
   <sheetData>
     <row r="1" spans="1:16" ht="23.4">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -471,7 +471,7 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -493,7 +493,7 @@
         <v>0.18254629629629629</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -508,34 +508,43 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="B5" s="6">
+        <v>4.1666666666666664E-2</v>
+      </c>
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="B6" s="6">
+        <v>2.0833333333333332E-2</v>
+      </c>
     </row>
     <row r="7" spans="1:16">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="B7" s="6">
+        <v>2.5694444444444447E-2</v>
       </c>
     </row>
     <row r="8" spans="1:16">
       <c r="A8" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:16">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:16">
       <c r="A10" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="6">
         <f>SUM(B3:B9)</f>
-        <v>0.25224537037037037</v>
+        <v>0.34043981481481483</v>
       </c>
     </row>
   </sheetData>

</xml_diff>